<commit_message>
Add 30 EMBA students (113 Shanghai class) to students.xlsx
Course5: 113C26501-113C26531, 6 groups from 113級上海班分組表

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/students.xlsx
+++ b/data/students.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E98"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1562,9 +1562,519 @@
         <v>114370244</v>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B69" t="str">
+        <v>113C26501</v>
+      </c>
+      <c r="C69" t="str">
+        <v>蔡彰哲</v>
+      </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
+      <c r="E69" t="str">
+        <v>113C26501</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B70" t="str">
+        <v>113C26502</v>
+      </c>
+      <c r="C70" t="str">
+        <v>朱文怡</v>
+      </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
+      <c r="E70" t="str">
+        <v>113C26502</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B71" t="str">
+        <v>113C26503</v>
+      </c>
+      <c r="C71" t="str">
+        <v>王光輝</v>
+      </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
+      <c r="E71" t="str">
+        <v>113C26503</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B72" t="str">
+        <v>113C26504</v>
+      </c>
+      <c r="C72" t="str">
+        <v>江明憲</v>
+      </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
+      <c r="E72" t="str">
+        <v>113C26504</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B73" t="str">
+        <v>113C26505</v>
+      </c>
+      <c r="C73" t="str">
+        <v>徐詩琴</v>
+      </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
+      <c r="E73" t="str">
+        <v>113C26505</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B74" t="str">
+        <v>113C26506</v>
+      </c>
+      <c r="C74" t="str">
+        <v>唐青文</v>
+      </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
+      <c r="E74" t="str">
+        <v>113C26506</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B75" t="str">
+        <v>113C26507</v>
+      </c>
+      <c r="C75" t="str">
+        <v>鄭昱暘</v>
+      </c>
+      <c r="D75" t="str">
+        <v/>
+      </c>
+      <c r="E75" t="str">
+        <v>113C26507</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B76" t="str">
+        <v>113C26508</v>
+      </c>
+      <c r="C76" t="str">
+        <v>曾任健</v>
+      </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
+      <c r="E76" t="str">
+        <v>113C26508</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B77" t="str">
+        <v>113C26509</v>
+      </c>
+      <c r="C77" t="str">
+        <v>鄧宇翔</v>
+      </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
+      <c r="E77" t="str">
+        <v>113C26509</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B78" t="str">
+        <v>113C26511</v>
+      </c>
+      <c r="C78" t="str">
+        <v>許志鴻</v>
+      </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
+      <c r="E78" t="str">
+        <v>113C26511</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B79" t="str">
+        <v>113C26512</v>
+      </c>
+      <c r="C79" t="str">
+        <v>陳佩宜</v>
+      </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
+      <c r="E79" t="str">
+        <v>113C26512</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B80" t="str">
+        <v>113C26513</v>
+      </c>
+      <c r="C80" t="str">
+        <v>廖倫群</v>
+      </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
+      <c r="E80" t="str">
+        <v>113C26513</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B81" t="str">
+        <v>113C26514</v>
+      </c>
+      <c r="C81" t="str">
+        <v>李後熙</v>
+      </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
+      <c r="E81" t="str">
+        <v>113C26514</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B82" t="str">
+        <v>113C26515</v>
+      </c>
+      <c r="C82" t="str">
+        <v>曾榮富</v>
+      </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
+      <c r="E82" t="str">
+        <v>113C26515</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B83" t="str">
+        <v>113C26516</v>
+      </c>
+      <c r="C83" t="str">
+        <v>巫大宇</v>
+      </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
+      <c r="E83" t="str">
+        <v>113C26516</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B84" t="str">
+        <v>113C26517</v>
+      </c>
+      <c r="C84" t="str">
+        <v>劉永霖</v>
+      </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
+      <c r="E84" t="str">
+        <v>113C26517</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B85" t="str">
+        <v>113C26518</v>
+      </c>
+      <c r="C85" t="str">
+        <v>顧國立</v>
+      </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
+      <c r="E85" t="str">
+        <v>113C26518</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B86" t="str">
+        <v>113C26519</v>
+      </c>
+      <c r="C86" t="str">
+        <v>盧仁傑</v>
+      </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
+      <c r="E86" t="str">
+        <v>113C26519</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B87" t="str">
+        <v>113C26520</v>
+      </c>
+      <c r="C87" t="str">
+        <v>魏明照</v>
+      </c>
+      <c r="D87" t="str">
+        <v/>
+      </c>
+      <c r="E87" t="str">
+        <v>113C26520</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B88" t="str">
+        <v>113C26521</v>
+      </c>
+      <c r="C88" t="str">
+        <v>陳勇廷</v>
+      </c>
+      <c r="D88" t="str">
+        <v/>
+      </c>
+      <c r="E88" t="str">
+        <v>113C26521</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B89" t="str">
+        <v>113C26522</v>
+      </c>
+      <c r="C89" t="str">
+        <v>陳麗玲</v>
+      </c>
+      <c r="D89" t="str">
+        <v/>
+      </c>
+      <c r="E89" t="str">
+        <v>113C26522</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B90" t="str">
+        <v>113C26523</v>
+      </c>
+      <c r="C90" t="str">
+        <v>楊光倫</v>
+      </c>
+      <c r="D90" t="str">
+        <v/>
+      </c>
+      <c r="E90" t="str">
+        <v>113C26523</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B91" t="str">
+        <v>113C26524</v>
+      </c>
+      <c r="C91" t="str">
+        <v>黃乙民</v>
+      </c>
+      <c r="D91" t="str">
+        <v/>
+      </c>
+      <c r="E91" t="str">
+        <v>113C26524</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B92" t="str">
+        <v>113C26525</v>
+      </c>
+      <c r="C92" t="str">
+        <v>姚昶志</v>
+      </c>
+      <c r="D92" t="str">
+        <v/>
+      </c>
+      <c r="E92" t="str">
+        <v>113C26525</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B93" t="str">
+        <v>113C26526</v>
+      </c>
+      <c r="C93" t="str">
+        <v>張瑋祥</v>
+      </c>
+      <c r="D93" t="str">
+        <v/>
+      </c>
+      <c r="E93" t="str">
+        <v>113C26526</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B94" t="str">
+        <v>113C26527</v>
+      </c>
+      <c r="C94" t="str">
+        <v>李菀頻</v>
+      </c>
+      <c r="D94" t="str">
+        <v/>
+      </c>
+      <c r="E94" t="str">
+        <v>113C26527</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B95" t="str">
+        <v>113C26528</v>
+      </c>
+      <c r="C95" t="str">
+        <v>陳穎婕</v>
+      </c>
+      <c r="D95" t="str">
+        <v/>
+      </c>
+      <c r="E95" t="str">
+        <v>113C26528</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B96" t="str">
+        <v>113C26529</v>
+      </c>
+      <c r="C96" t="str">
+        <v>許育銘</v>
+      </c>
+      <c r="D96" t="str">
+        <v/>
+      </c>
+      <c r="E96" t="str">
+        <v>113C26529</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B97" t="str">
+        <v>113C26530</v>
+      </c>
+      <c r="C97" t="str">
+        <v>王子欣</v>
+      </c>
+      <c r="D97" t="str">
+        <v/>
+      </c>
+      <c r="E97" t="str">
+        <v>113C26530</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B98" t="str">
+        <v>113C26531</v>
+      </c>
+      <c r="C98" t="str">
+        <v>邱明加</v>
+      </c>
+      <c r="D98" t="str">
+        <v/>
+      </c>
+      <c r="E98" t="str">
+        <v>113C26531</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E68"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E98"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>